<commit_message>
Restore MesDiagnosticReport profile details 5405eb9d8f9163968fb1a9cd02db5034766c86bc
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-mesures-diagnostic-report.xlsx
+++ b/main/ig/StructureDefinition-mesures-diagnostic-report.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1464" uniqueCount="353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1464" uniqueCount="354">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-02T08:10:43+00:00</t>
+    <t>2026-02-02T09:29:40+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -930,6 +930,10 @@
   </si>
   <si>
     <t>trigly-cholesterol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference(https://interop.esante.gouv.fr/ig/fhir/mesures/StructureDefinition/mesures-observation-cholesterol-trigly)
+</t>
   </si>
   <si>
     <t>DiagnosticReport.result:cholesterol-aspect</t>
@@ -4521,7 +4525,7 @@
         <v>80</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>269</v>
+        <v>289</v>
       </c>
       <c r="L27" t="s" s="2">
         <v>270</v>
@@ -4611,13 +4615,13 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B28" t="s" s="2">
         <v>267</v>
       </c>
       <c r="C28" t="s" s="2">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D28" t="s" s="2">
         <v>268</v>
@@ -4639,7 +4643,7 @@
         <v>80</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L28" t="s" s="2">
         <v>270</v>
@@ -4729,13 +4733,13 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B29" t="s" s="2">
         <v>267</v>
       </c>
       <c r="C29" t="s" s="2">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D29" t="s" s="2">
         <v>268</v>
@@ -4757,7 +4761,7 @@
         <v>80</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="L29" t="s" s="2">
         <v>270</v>
@@ -4847,10 +4851,10 @@
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -4873,16 +4877,16 @@
         <v>80</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="N30" t="s" s="2">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
@@ -4932,7 +4936,7 @@
         <v>80</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>78</v>
@@ -4953,7 +4957,7 @@
         <v>80</v>
       </c>
       <c r="AM30" t="s" s="2">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="AN30" t="s" s="2">
         <v>80</v>
@@ -4961,14 +4965,14 @@
     </row>
     <row r="31" hidden="true">
       <c r="A31" t="s" s="2">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s" s="2">
@@ -4987,17 +4991,17 @@
         <v>91</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="N31" s="2"/>
       <c r="O31" t="s" s="2">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="P31" t="s" s="2">
         <v>80</v>
@@ -5046,7 +5050,7 @@
         <v>80</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>78</v>
@@ -5064,7 +5068,7 @@
         <v>80</v>
       </c>
       <c r="AL31" t="s" s="2">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="AM31" t="s" s="2">
         <v>277</v>
@@ -5075,10 +5079,10 @@
     </row>
     <row r="32" hidden="true">
       <c r="A32" t="s" s="2">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -5101,13 +5105,13 @@
         <v>80</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -5158,7 +5162,7 @@
         <v>80</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>78</v>
@@ -5179,7 +5183,7 @@
         <v>80</v>
       </c>
       <c r="AM32" t="s" s="2">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="AN32" t="s" s="2">
         <v>80</v>
@@ -5187,10 +5191,10 @@
     </row>
     <row r="33" hidden="true">
       <c r="A33" t="s" s="2">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5219,7 +5223,7 @@
         <v>137</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="N33" t="s" s="2">
         <v>139</v>
@@ -5272,7 +5276,7 @@
         <v>80</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>78</v>
@@ -5293,7 +5297,7 @@
         <v>80</v>
       </c>
       <c r="AM33" t="s" s="2">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="AN33" t="s" s="2">
         <v>80</v>
@@ -5301,14 +5305,14 @@
     </row>
     <row r="34" hidden="true">
       <c r="A34" t="s" s="2">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" t="s" s="2">
@@ -5330,10 +5334,10 @@
         <v>136</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="N34" t="s" s="2">
         <v>139</v>
@@ -5388,7 +5392,7 @@
         <v>80</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>78</v>
@@ -5417,10 +5421,10 @@
     </row>
     <row r="35" hidden="true">
       <c r="A35" t="s" s="2">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5443,19 +5447,19 @@
         <v>80</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="N35" t="s" s="2">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="O35" t="s" s="2">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="P35" t="s" s="2">
         <v>80</v>
@@ -5504,7 +5508,7 @@
         <v>80</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>78</v>
@@ -5525,7 +5529,7 @@
         <v>80</v>
       </c>
       <c r="AM35" t="s" s="2">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="AN35" t="s" s="2">
         <v>80</v>
@@ -5533,10 +5537,10 @@
     </row>
     <row r="36" hidden="true">
       <c r="A36" t="s" s="2">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5559,13 +5563,13 @@
         <v>91</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
@@ -5616,7 +5620,7 @@
         <v>80</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>90</v>
@@ -5637,7 +5641,7 @@
         <v>80</v>
       </c>
       <c r="AM36" t="s" s="2">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="AN36" t="s" s="2">
         <v>80</v>
@@ -5645,14 +5649,14 @@
     </row>
     <row r="37" hidden="true">
       <c r="A37" t="s" s="2">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" t="s" s="2">
@@ -5671,17 +5675,17 @@
         <v>80</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="N37" s="2"/>
       <c r="O37" t="s" s="2">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="P37" t="s" s="2">
         <v>80</v>
@@ -5730,7 +5734,7 @@
         <v>80</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>78</v>
@@ -5748,10 +5752,10 @@
         <v>80</v>
       </c>
       <c r="AL37" t="s" s="2">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="AM37" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="AN37" t="s" s="2">
         <v>80</v>
@@ -5759,10 +5763,10 @@
     </row>
     <row r="38" hidden="true">
       <c r="A38" t="s" s="2">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -5788,10 +5792,10 @@
         <v>180</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
@@ -5821,10 +5825,10 @@
         <v>184</v>
       </c>
       <c r="Y38" t="s" s="2">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="Z38" t="s" s="2">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="AA38" t="s" s="2">
         <v>80</v>
@@ -5842,7 +5846,7 @@
         <v>80</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>78</v>
@@ -5860,10 +5864,10 @@
         <v>80</v>
       </c>
       <c r="AL38" t="s" s="2">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="AM38" t="s" s="2">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="AN38" t="s" s="2">
         <v>80</v>
@@ -5871,10 +5875,10 @@
     </row>
     <row r="39" hidden="true">
       <c r="A39" t="s" s="2">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5897,19 +5901,19 @@
         <v>80</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="N39" t="s" s="2">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="O39" t="s" s="2">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="P39" t="s" s="2">
         <v>80</v>
@@ -5958,7 +5962,7 @@
         <v>80</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>78</v>
@@ -5976,10 +5980,10 @@
         <v>80</v>
       </c>
       <c r="AL39" t="s" s="2">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="AM39" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="AN39" t="s" s="2">
         <v>80</v>

</xml_diff>